<commit_message>
vault backup: 2026-03-17 15:35:36
</commit_message>
<xml_diff>
--- a/BWL/Übung/Übungen/UE01b/BWL2T2_02_UE01b_Betriebsüberleitungsbogen (Vorlage).xlsx
+++ b/BWL/Übung/Übungen/UE01b/BWL2T2_02_UE01b_Betriebsüberleitungsbogen (Vorlage).xlsx
@@ -262,7 +262,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="1" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -299,6 +299,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf fontId="4" fillId="4" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -799,7 +803,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="33.7109375"/>
-    <col customWidth="1" min="2" max="2" width="22"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" width="23.453125"/>
     <col customWidth="1" min="3" max="3" width="19.85546875"/>
     <col customWidth="1" min="4" max="4" width="19.28515625"/>
     <col customWidth="1" min="5" max="5" width="19.85546875"/>
@@ -997,13 +1001,13 @@
         <v>20</v>
       </c>
       <c r="B12" s="9">
-        <v>0</v>
+        <v>422</v>
       </c>
       <c r="C12" s="9">
         <v>960</v>
       </c>
       <c r="D12" s="9">
-        <v>0</v>
+        <v>422</v>
       </c>
       <c r="E12" s="9">
         <f>12000*0.08</f>
@@ -1036,7 +1040,7 @@
       </c>
       <c r="B14" s="15">
         <f>SUM(B4:B13)</f>
-        <v>1664</v>
+        <v>2086</v>
       </c>
       <c r="C14" s="15"/>
       <c r="D14" s="15"/>
@@ -1046,6 +1050,19 @@
       </c>
     </row>
     <row r="15" ht="15.75"/>
+    <row r="28" ht="14.25">
+      <c r="B28" s="16"/>
+    </row>
+    <row r="47" ht="14.25">
+      <c r="B47" s="17"/>
+    </row>
+    <row r="52" ht="14.25">
+      <c r="B52" s="16"/>
+    </row>
+    <row r="63" ht="14.25">
+      <c r="B63" s="17"/>
+      <c r="C63" s="17"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:A3"/>

</xml_diff>